<commit_message>
feat: complete interactive roadmap, role-based dashboards, database query retry, and dynamic email links
</commit_message>
<xml_diff>
--- a/Yantriksha_X_Hub_Project_Checklist.xlsx
+++ b/Yantriksha_X_Hub_Project_Checklist.xlsx
@@ -552,7 +552,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -576,7 +575,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -765,7 +764,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -792,7 +791,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -819,7 +818,7 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -846,7 +845,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -873,7 +872,7 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -900,7 +899,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -927,7 +926,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -954,7 +953,7 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1034,7 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1061,7 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1088,7 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1115,7 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1142,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1250,7 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1277,7 @@
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1304,7 @@
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1331,7 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1358,7 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1385,7 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1412,7 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1439,7 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1466,7 @@
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1493,7 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1520,7 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1547,7 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>